<commit_message>
Fix formula-error validation check
Replaced the placeholder formula-error result with a formula that counts actual errors across the calculated model ranges. Verified that the check changes to FAIL when an error is introduced and returns to PASS after the formula is restored.
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jaylozano/Documents/Codex/2026-09-02/bus/outputs/final/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCBE04EF-37F4-6042-9A8C-B29B30186910}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE39AC62-2468-2E41-9788-8463CD32A270}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1660" yWindow="1060" windowWidth="44800" windowHeight="23260" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22320" yWindow="600" windowWidth="22480" windowHeight="23240" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
@@ -127,6 +127,28 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -903,11 +925,11 @@
     <xf numFmtId="164" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1174,7 +1196,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15" customHeight="1">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="21"/>
@@ -1182,7 +1204,7 @@
       <c r="D1" s="21"/>
     </row>
     <row r="2" spans="1:4" ht="24" customHeight="1">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="21"/>
@@ -1546,7 +1568,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15" customHeight="1">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="22" t="s">
         <v>42</v>
       </c>
       <c r="B1" s="21"/>
@@ -1554,7 +1576,7 @@
       <c r="D1" s="21"/>
     </row>
     <row r="2" spans="1:4" ht="24" customHeight="1">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="20" t="s">
         <v>43</v>
       </c>
       <c r="B2" s="21"/>
@@ -1826,7 +1848,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="15" customHeight="1">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="22" t="s">
         <v>78</v>
       </c>
       <c r="B1" s="21"/>
@@ -1853,7 +1875,7 @@
       <c r="W1" s="21"/>
     </row>
     <row r="2" spans="1:23" ht="15" customHeight="1">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="20" t="s">
         <v>79</v>
       </c>
       <c r="B2" s="21"/>
@@ -4228,7 +4250,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15" customHeight="1">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="22" t="s">
         <v>90</v>
       </c>
       <c r="B1" s="21"/>
@@ -4237,7 +4259,7 @@
       <c r="E1" s="21"/>
     </row>
     <row r="2" spans="1:5" ht="24" customHeight="1">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="20" t="s">
         <v>91</v>
       </c>
       <c r="B2" s="21"/>
@@ -4606,7 +4628,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15" customHeight="1">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="22" t="s">
         <v>124</v>
       </c>
       <c r="B1" s="21"/>
@@ -4617,7 +4639,7 @@
       <c r="G1" s="2"/>
     </row>
     <row r="2" spans="1:7" ht="24" customHeight="1">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="20" t="s">
         <v>125</v>
       </c>
       <c r="B2" s="21"/>
@@ -5066,8 +5088,8 @@
       <c r="A22" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="B22" s="18">
-        <f>0</f>
+      <c r="B22" s="18" cm="1">
+        <f t="array" ref="B22">SUMPRODUCT(--ISERROR('Cost Structure'!B4:B18))+SUMPRODUCT(--ISERROR('Marginal-Cost Schedules'!B5:W35))+SUMPRODUCT(--ISERROR(Optimization!B10:B28))</f>
         <v>0</v>
       </c>
       <c r="C22" s="3" t="s">

</xml_diff>